<commit_message>
Show game type instead of date/location in games table
</commit_message>
<xml_diff>
--- a/data/raw_games/11U Spring 2026/Games.xlsx
+++ b/data/raw_games/11U Spring 2026/Games.xlsx
@@ -1449,6 +1449,15 @@
   </si>
   <si>
     <t>Grapevine</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Pool</t>
+  </si>
+  <si>
+    <t>Bracket</t>
   </si>
 </sst>
 </file>
@@ -1830,10 +1839,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <cols>
-    <col min="4" max="4" width="37.82" customWidth="1"/>
-    <col min="5" max="5" width="11.74" customWidth="1"/>
-    <col min="6" max="6" width="31.35" customWidth="1"/>
-    <col min="7" max="7" width="12.65" customWidth="1"/>
+    <col min="5" max="5" width="37.82" customWidth="1"/>
+    <col min="6" max="6" width="11.74" customWidth="1"/>
+    <col min="7" max="7" width="31.35" customWidth="1"/>
+    <col min="8" max="8" width="12.65" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1841,27 +1850,30 @@
         <v>345</v>
       </c>
       <c r="B2" s="0" t="s">
+        <v>470</v>
+      </c>
+      <c r="C2" s="0" t="s">
         <v>346</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="D2" s="0" t="s">
         <v>452</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="E2" s="0" t="s">
         <v>366</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="F2" s="0" t="s">
         <v>370</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="G2" s="0" t="s">
         <v>367</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="H2" s="0" t="s">
         <v>371</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="I2" s="0" t="s">
         <v>349</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="J2" s="0" t="s">
         <v>383</v>
       </c>
     </row>
@@ -1870,27 +1882,30 @@
         <v>46081</v>
       </c>
       <c r="B3" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C3" s="0" t="s">
         <v>448</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="D3" s="0" t="s">
         <v>453</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="E3" s="0" t="s">
         <v>350</v>
       </c>
-      <c r="E3" s="0">
+      <c r="F3" s="0">
         <v>9</v>
       </c>
-      <c r="F3" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G3" s="0">
+      <c r="G3" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H3" s="0">
         <v>10</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="I3" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="J3" s="0" t="s">
         <v>384</v>
       </c>
     </row>
@@ -1899,27 +1914,30 @@
         <v>46081</v>
       </c>
       <c r="B4" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C4" s="0" t="s">
         <v>448</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="D4" s="0" t="s">
         <v>453</v>
       </c>
-      <c r="D4" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E4" s="0">
+      <c r="E4" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F4" s="0">
         <v>0</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="G4" s="0" t="s">
         <v>355</v>
       </c>
-      <c r="G4" s="0">
+      <c r="H4" s="0">
         <v>12</v>
       </c>
-      <c r="H4" s="0" t="s">
+      <c r="I4" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="J4" s="0" t="s">
         <v>385</v>
       </c>
     </row>
@@ -1928,27 +1946,30 @@
         <v>46082</v>
       </c>
       <c r="B5" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C5" s="0" t="s">
         <v>448</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="D5" s="0" t="s">
         <v>453</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="E5" s="0" t="s">
         <v>354</v>
       </c>
-      <c r="E5" s="0">
+      <c r="F5" s="0">
         <v>10</v>
       </c>
-      <c r="F5" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G5" s="0">
+      <c r="G5" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H5" s="0">
         <v>9</v>
       </c>
-      <c r="H5" s="0" t="s">
+      <c r="I5" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I5" s="0" t="s">
+      <c r="J5" s="0" t="s">
         <v>386</v>
       </c>
     </row>
@@ -1957,27 +1978,30 @@
         <v>46102</v>
       </c>
       <c r="B6" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C6" s="0" t="s">
         <v>451</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="D6" s="0" t="s">
         <v>454</v>
       </c>
-      <c r="D6" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E6" s="0">
+      <c r="E6" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F6" s="0">
         <v>15</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="G6" s="0" t="s">
         <v>358</v>
       </c>
-      <c r="G6" s="0">
+      <c r="H6" s="0">
         <v>3</v>
       </c>
-      <c r="H6" s="0" t="s">
+      <c r="I6" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I6" s="0" t="s">
+      <c r="J6" s="0" t="s">
         <v>387</v>
       </c>
     </row>
@@ -1986,27 +2010,30 @@
         <v>46102</v>
       </c>
       <c r="B7" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C7" s="0" t="s">
         <v>451</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="D7" s="0" t="s">
         <v>454</v>
       </c>
-      <c r="D7" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E7" s="0">
+      <c r="E7" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F7" s="0">
         <v>8</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="G7" s="0" t="s">
         <v>361</v>
       </c>
-      <c r="G7" s="0">
+      <c r="H7" s="0">
         <v>6</v>
       </c>
-      <c r="H7" s="0" t="s">
+      <c r="I7" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I7" s="0" t="s">
+      <c r="J7" s="0" t="s">
         <v>388</v>
       </c>
     </row>
@@ -2015,27 +2042,30 @@
         <v>46103</v>
       </c>
       <c r="B8" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C8" s="0" t="s">
         <v>451</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="D8" s="0" t="s">
         <v>454</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="E8" s="0" t="s">
         <v>364</v>
       </c>
-      <c r="E8" s="0">
+      <c r="F8" s="0">
         <v>7</v>
       </c>
-      <c r="F8" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G8" s="0">
+      <c r="G8" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H8" s="0">
         <v>8</v>
       </c>
-      <c r="H8" s="0" t="s">
+      <c r="I8" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I8" s="0" t="s">
+      <c r="J8" s="0" t="s">
         <v>389</v>
       </c>
     </row>
@@ -2044,27 +2074,30 @@
         <v>46103</v>
       </c>
       <c r="B9" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C9" s="0" t="s">
         <v>451</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="D9" s="0" t="s">
         <v>454</v>
       </c>
-      <c r="D9" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E9" s="0">
+      <c r="E9" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F9" s="0">
         <v>3</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="G9" s="0" t="s">
         <v>361</v>
       </c>
-      <c r="G9" s="0">
+      <c r="H9" s="0">
         <v>1</v>
       </c>
-      <c r="H9" s="0" t="s">
+      <c r="I9" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I9" s="0" t="s">
+      <c r="J9" s="0" t="s">
         <v>390</v>
       </c>
     </row>
@@ -2073,27 +2106,30 @@
         <v>46103</v>
       </c>
       <c r="B10" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C10" s="0" t="s">
         <v>451</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="D10" s="0" t="s">
         <v>454</v>
       </c>
-      <c r="D10" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E10" s="0">
+      <c r="E10" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F10" s="0">
         <v>1</v>
       </c>
-      <c r="F10" s="0" t="s">
+      <c r="G10" s="0" t="s">
         <v>358</v>
       </c>
-      <c r="G10" s="0">
+      <c r="H10" s="0">
         <v>9</v>
       </c>
-      <c r="H10" s="0" t="s">
+      <c r="I10" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I10" s="0" t="s">
+      <c r="J10" s="0" t="s">
         <v>391</v>
       </c>
     </row>
@@ -2102,27 +2138,30 @@
         <v>46109</v>
       </c>
       <c r="B11" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C11" s="0" t="s">
         <v>455</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="D11" s="0" t="s">
         <v>456</v>
       </c>
-      <c r="D11" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E11" s="0">
+      <c r="E11" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F11" s="0">
         <v>13</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="G11" s="0" t="s">
         <v>376</v>
       </c>
-      <c r="G11" s="0">
+      <c r="H11" s="0">
         <v>1</v>
       </c>
-      <c r="H11" s="0" t="s">
+      <c r="I11" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I11" s="0" t="s">
+      <c r="J11" s="0" t="s">
         <v>392</v>
       </c>
     </row>
@@ -2131,27 +2170,30 @@
         <v>46109</v>
       </c>
       <c r="B12" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C12" s="0" t="s">
         <v>455</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="D12" s="0" t="s">
         <v>456</v>
       </c>
-      <c r="D12" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E12" s="0">
+      <c r="E12" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F12" s="0">
         <v>15</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="G12" s="0" t="s">
         <v>377</v>
       </c>
-      <c r="G12" s="0">
+      <c r="H12" s="0">
         <v>0</v>
       </c>
-      <c r="H12" s="0" t="s">
+      <c r="I12" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I12" s="0" t="s">
+      <c r="J12" s="0" t="s">
         <v>393</v>
       </c>
     </row>
@@ -2160,27 +2202,30 @@
         <v>46110</v>
       </c>
       <c r="B13" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C13" s="0" t="s">
         <v>455</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="D13" s="0" t="s">
         <v>456</v>
       </c>
-      <c r="D13" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E13" s="0">
+      <c r="E13" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F13" s="0">
         <v>7</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="G13" s="0" t="s">
         <v>361</v>
       </c>
-      <c r="G13" s="0">
+      <c r="H13" s="0">
         <v>6</v>
       </c>
-      <c r="H13" s="0" t="s">
+      <c r="I13" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I13" s="0" t="s">
+      <c r="J13" s="0" t="s">
         <v>394</v>
       </c>
     </row>
@@ -2189,27 +2234,30 @@
         <v>46110</v>
       </c>
       <c r="B14" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C14" s="0" t="s">
         <v>455</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="D14" s="0" t="s">
         <v>456</v>
       </c>
-      <c r="D14" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E14" s="0">
+      <c r="E14" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F14" s="0">
         <v>9</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="G14" s="0" t="s">
         <v>379</v>
       </c>
-      <c r="G14" s="0">
+      <c r="H14" s="0">
         <v>2</v>
       </c>
-      <c r="H14" s="0" t="s">
+      <c r="I14" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I14" s="0" t="s">
+      <c r="J14" s="0" t="s">
         <v>395</v>
       </c>
     </row>
@@ -2218,27 +2266,30 @@
         <v>46123</v>
       </c>
       <c r="B15" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C15" s="0" t="s">
         <v>458</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="D15" s="0" t="s">
         <v>459</v>
       </c>
-      <c r="D15" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E15" s="0">
+      <c r="E15" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F15" s="0">
         <v>15</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="G15" s="0" t="s">
         <v>380</v>
       </c>
-      <c r="G15" s="0">
+      <c r="H15" s="0">
         <v>6</v>
       </c>
-      <c r="H15" s="0" t="s">
+      <c r="I15" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I15" s="0" t="s">
+      <c r="J15" s="0" t="s">
         <v>396</v>
       </c>
     </row>
@@ -2247,27 +2298,30 @@
         <v>46123</v>
       </c>
       <c r="B16" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C16" s="0" t="s">
         <v>458</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="D16" s="0" t="s">
         <v>459</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="E16" s="0" t="s">
         <v>381</v>
       </c>
-      <c r="E16" s="0">
+      <c r="F16" s="0">
         <v>7</v>
       </c>
-      <c r="F16" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G16" s="0">
+      <c r="G16" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H16" s="0">
         <v>4</v>
       </c>
-      <c r="H16" s="0" t="s">
+      <c r="I16" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I16" s="0" t="s">
+      <c r="J16" s="0" t="s">
         <v>398</v>
       </c>
     </row>
@@ -2276,27 +2330,30 @@
         <v>46136</v>
       </c>
       <c r="B17" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C17" s="0" t="s">
         <v>460</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="D17" s="0" t="s">
         <v>461</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="E17" s="0" t="s">
         <v>399</v>
       </c>
-      <c r="E17" s="0">
+      <c r="F17" s="0">
         <v>9</v>
       </c>
-      <c r="F17" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G17" s="0">
+      <c r="G17" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H17" s="0">
         <v>1</v>
       </c>
-      <c r="H17" s="0" t="s">
+      <c r="I17" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I17" s="0" t="s">
+      <c r="J17" s="0" t="s">
         <v>400</v>
       </c>
     </row>
@@ -2305,27 +2362,30 @@
         <v>46136</v>
       </c>
       <c r="B18" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C18" s="0" t="s">
         <v>460</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="D18" s="0" t="s">
         <v>461</v>
       </c>
-      <c r="D18" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E18" s="0">
+      <c r="E18" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F18" s="0">
         <v>3</v>
       </c>
-      <c r="F18" s="0" t="s">
+      <c r="G18" s="0" t="s">
         <v>401</v>
       </c>
-      <c r="G18" s="0">
+      <c r="H18" s="0">
         <v>9</v>
       </c>
-      <c r="H18" s="0" t="s">
+      <c r="I18" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I18" s="0" t="s">
+      <c r="J18" s="0" t="s">
         <v>402</v>
       </c>
     </row>
@@ -2334,27 +2394,30 @@
         <v>46138</v>
       </c>
       <c r="B19" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C19" s="0" t="s">
         <v>460</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="D19" s="0" t="s">
         <v>461</v>
       </c>
-      <c r="D19" s="0" t="s">
+      <c r="E19" s="0" t="s">
         <v>403</v>
       </c>
-      <c r="E19" s="0">
+      <c r="F19" s="0">
         <v>7</v>
       </c>
-      <c r="F19" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G19" s="0">
+      <c r="G19" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H19" s="0">
         <v>1</v>
       </c>
-      <c r="H19" s="0" t="s">
+      <c r="I19" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I19" s="0" t="s">
+      <c r="J19" s="0" t="s">
         <v>404</v>
       </c>
     </row>
@@ -2363,27 +2426,30 @@
         <v>46144</v>
       </c>
       <c r="B20" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C20" s="0" t="s">
         <v>462</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="D20" s="0" t="s">
         <v>459</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="E20" s="0" t="s">
         <v>406</v>
       </c>
-      <c r="E20" s="0">
+      <c r="F20" s="0">
         <v>15</v>
       </c>
-      <c r="F20" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G20" s="0">
+      <c r="G20" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H20" s="0">
         <v>1</v>
       </c>
-      <c r="H20" s="0" t="s">
+      <c r="I20" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I20" s="0" t="s">
+      <c r="J20" s="0" t="s">
         <v>407</v>
       </c>
     </row>
@@ -2392,27 +2458,30 @@
         <v>46144</v>
       </c>
       <c r="B21" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C21" s="0" t="s">
         <v>462</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="D21" s="0" t="s">
         <v>459</v>
       </c>
-      <c r="D21" s="0" t="s">
+      <c r="E21" s="0" t="s">
         <v>408</v>
       </c>
-      <c r="E21" s="0">
+      <c r="F21" s="0">
         <v>6</v>
       </c>
-      <c r="F21" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G21" s="0">
+      <c r="G21" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H21" s="0">
         <v>5</v>
       </c>
-      <c r="H21" s="0" t="s">
+      <c r="I21" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I21" s="0" t="s">
+      <c r="J21" s="0" t="s">
         <v>351</v>
       </c>
     </row>
@@ -2421,27 +2490,30 @@
         <v>46145</v>
       </c>
       <c r="B22" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C22" s="0" t="s">
         <v>462</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="D22" s="0" t="s">
         <v>459</v>
       </c>
-      <c r="D22" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E22" s="0">
+      <c r="E22" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F22" s="0">
         <v>13</v>
       </c>
-      <c r="F22" s="0" t="s">
+      <c r="G22" s="0" t="s">
         <v>409</v>
       </c>
-      <c r="G22" s="0">
+      <c r="H22" s="0">
         <v>15</v>
       </c>
-      <c r="H22" s="0" t="s">
+      <c r="I22" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I22" s="0" t="s">
+      <c r="J22" s="0" t="s">
         <v>410</v>
       </c>
     </row>
@@ -2450,27 +2522,30 @@
         <v>46158</v>
       </c>
       <c r="B23" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C23" s="0" t="s">
         <v>464</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="D23" s="0" t="s">
         <v>453</v>
       </c>
-      <c r="D23" s="0" t="s">
+      <c r="E23" s="0" t="s">
         <v>411</v>
       </c>
-      <c r="E23" s="0">
+      <c r="F23" s="0">
         <v>11</v>
       </c>
-      <c r="F23" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G23" s="0">
+      <c r="G23" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H23" s="0">
         <v>4</v>
       </c>
-      <c r="H23" s="0" t="s">
+      <c r="I23" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I23" s="0" t="s">
+      <c r="J23" s="0" t="s">
         <v>412</v>
       </c>
     </row>
@@ -2479,27 +2554,30 @@
         <v>46158</v>
       </c>
       <c r="B24" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C24" s="0" t="s">
         <v>464</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="D24" s="0" t="s">
         <v>453</v>
       </c>
-      <c r="D24" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E24" s="0">
+      <c r="E24" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F24" s="0">
         <v>3</v>
       </c>
-      <c r="F24" s="0" t="s">
+      <c r="G24" s="0" t="s">
         <v>413</v>
       </c>
-      <c r="G24" s="0">
+      <c r="H24" s="0">
         <v>15</v>
       </c>
-      <c r="H24" s="0" t="s">
+      <c r="I24" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I24" s="0" t="s">
+      <c r="J24" s="0" t="s">
         <v>414</v>
       </c>
     </row>
@@ -2508,27 +2586,30 @@
         <v>46159</v>
       </c>
       <c r="B25" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C25" s="0" t="s">
         <v>464</v>
       </c>
-      <c r="C25" s="0" t="s">
+      <c r="D25" s="0" t="s">
         <v>453</v>
       </c>
-      <c r="D25" s="0" t="s">
+      <c r="E25" s="0" t="s">
         <v>415</v>
       </c>
-      <c r="E25" s="0">
+      <c r="F25" s="0">
         <v>8</v>
       </c>
-      <c r="F25" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G25" s="0">
+      <c r="G25" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H25" s="0">
         <v>0</v>
       </c>
-      <c r="H25" s="0" t="s">
+      <c r="I25" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I25" s="0" t="s">
+      <c r="J25" s="0" t="s">
         <v>416</v>
       </c>
     </row>
@@ -2537,27 +2618,30 @@
         <v>46165</v>
       </c>
       <c r="B26" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C26" s="0" t="s">
         <v>465</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="D26" s="0" t="s">
         <v>453</v>
       </c>
-      <c r="D26" s="0" t="s">
+      <c r="E26" s="0" t="s">
         <v>417</v>
       </c>
-      <c r="E26" s="0">
+      <c r="F26" s="0">
         <v>16</v>
       </c>
-      <c r="F26" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G26" s="0">
+      <c r="G26" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H26" s="0">
         <v>5</v>
       </c>
-      <c r="H26" s="0" t="s">
+      <c r="I26" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I26" s="0" t="s">
+      <c r="J26" s="0" t="s">
         <v>418</v>
       </c>
     </row>
@@ -2566,27 +2650,30 @@
         <v>46165</v>
       </c>
       <c r="B27" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C27" s="0" t="s">
         <v>465</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="D27" s="0" t="s">
         <v>453</v>
       </c>
-      <c r="D27" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E27" s="0">
+      <c r="E27" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F27" s="0">
         <v>9</v>
       </c>
-      <c r="F27" s="0" t="s">
+      <c r="G27" s="0" t="s">
         <v>422</v>
       </c>
-      <c r="G27" s="0">
+      <c r="H27" s="0">
         <v>7</v>
       </c>
-      <c r="H27" s="0" t="s">
+      <c r="I27" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I27" s="0" t="s">
+      <c r="J27" s="0" t="s">
         <v>419</v>
       </c>
     </row>
@@ -2595,27 +2682,30 @@
         <v>46166</v>
       </c>
       <c r="B28" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C28" s="0" t="s">
         <v>465</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="D28" s="0" t="s">
         <v>453</v>
       </c>
-      <c r="D28" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E28" s="0">
+      <c r="E28" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F28" s="0">
         <v>12</v>
       </c>
-      <c r="F28" s="0" t="s">
+      <c r="G28" s="0" t="s">
         <v>422</v>
       </c>
-      <c r="G28" s="0">
+      <c r="H28" s="0">
         <v>5</v>
       </c>
-      <c r="H28" s="0" t="s">
+      <c r="I28" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I28" s="0" t="s">
+      <c r="J28" s="0" t="s">
         <v>420</v>
       </c>
     </row>
@@ -2624,27 +2714,30 @@
         <v>46166</v>
       </c>
       <c r="B29" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C29" s="0" t="s">
         <v>465</v>
       </c>
-      <c r="C29" s="0" t="s">
+      <c r="D29" s="0" t="s">
         <v>453</v>
       </c>
-      <c r="D29" s="0" t="s">
+      <c r="E29" s="0" t="s">
         <v>423</v>
       </c>
-      <c r="E29" s="0">
+      <c r="F29" s="0">
         <v>8</v>
       </c>
-      <c r="F29" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G29" s="0">
+      <c r="G29" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H29" s="0">
         <v>0</v>
       </c>
-      <c r="H29" s="0" t="s">
+      <c r="I29" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I29" s="0" t="s">
+      <c r="J29" s="0" t="s">
         <v>421</v>
       </c>
     </row>
@@ -2653,27 +2746,30 @@
         <v>46179</v>
       </c>
       <c r="B30" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C30" s="0" t="s">
         <v>466</v>
       </c>
-      <c r="C30" s="0" t="s">
+      <c r="D30" s="0" t="s">
         <v>467</v>
       </c>
-      <c r="D30" s="0" t="s">
+      <c r="E30" s="0" t="s">
         <v>424</v>
       </c>
-      <c r="E30" s="0">
+      <c r="F30" s="0">
         <v>4</v>
       </c>
-      <c r="F30" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G30" s="0">
+      <c r="G30" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H30" s="0">
         <v>9</v>
       </c>
-      <c r="H30" s="0" t="s">
+      <c r="I30" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I30" s="0" t="s">
+      <c r="J30" s="0" t="s">
         <v>425</v>
       </c>
     </row>
@@ -2682,27 +2778,30 @@
         <v>46179</v>
       </c>
       <c r="B31" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C31" s="0" t="s">
         <v>466</v>
       </c>
-      <c r="C31" s="0" t="s">
+      <c r="D31" s="0" t="s">
         <v>467</v>
       </c>
-      <c r="D31" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E31" s="0">
+      <c r="E31" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F31" s="0">
         <v>6</v>
       </c>
-      <c r="F31" s="0" t="s">
+      <c r="G31" s="0" t="s">
         <v>430</v>
       </c>
-      <c r="G31" s="0">
+      <c r="H31" s="0">
         <v>8</v>
       </c>
-      <c r="H31" s="0" t="s">
+      <c r="I31" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I31" s="0" t="s">
+      <c r="J31" s="0" t="s">
         <v>426</v>
       </c>
     </row>
@@ -2711,27 +2810,30 @@
         <v>46180</v>
       </c>
       <c r="B32" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C32" s="0" t="s">
         <v>466</v>
       </c>
-      <c r="C32" s="0" t="s">
+      <c r="D32" s="0" t="s">
         <v>467</v>
       </c>
-      <c r="D32" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E32" s="0">
+      <c r="E32" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F32" s="0">
         <v>17</v>
       </c>
-      <c r="F32" s="0" t="s">
+      <c r="G32" s="0" t="s">
         <v>431</v>
       </c>
-      <c r="G32" s="0">
+      <c r="H32" s="0">
         <v>4</v>
       </c>
-      <c r="H32" s="0" t="s">
+      <c r="I32" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I32" s="0" t="s">
+      <c r="J32" s="0" t="s">
         <v>427</v>
       </c>
     </row>
@@ -2740,27 +2842,30 @@
         <v>46180</v>
       </c>
       <c r="B33" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C33" s="0" t="s">
         <v>466</v>
       </c>
-      <c r="C33" s="0" t="s">
+      <c r="D33" s="0" t="s">
         <v>467</v>
       </c>
-      <c r="D33" s="0" t="s">
+      <c r="E33" s="0" t="s">
         <v>430</v>
       </c>
-      <c r="E33" s="0">
+      <c r="F33" s="0">
         <v>9</v>
       </c>
-      <c r="F33" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G33" s="0">
+      <c r="G33" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H33" s="0">
         <v>2</v>
       </c>
-      <c r="H33" s="0" t="s">
+      <c r="I33" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I33" s="0" t="s">
+      <c r="J33" s="0" t="s">
         <v>428</v>
       </c>
     </row>
@@ -2769,27 +2874,30 @@
         <v>46193</v>
       </c>
       <c r="B34" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C34" s="0" t="s">
         <v>468</v>
       </c>
-      <c r="C34" s="0" t="s">
+      <c r="D34" s="0" t="s">
         <v>469</v>
       </c>
-      <c r="D34" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E34" s="0">
+      <c r="E34" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F34" s="0">
         <v>10</v>
       </c>
-      <c r="F34" s="0" t="s">
+      <c r="G34" s="0" t="s">
         <v>432</v>
       </c>
-      <c r="G34" s="0">
+      <c r="H34" s="0">
         <v>15</v>
       </c>
-      <c r="H34" s="0" t="s">
+      <c r="I34" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I34" s="0" t="s">
+      <c r="J34" s="0" t="s">
         <v>434</v>
       </c>
     </row>
@@ -2798,27 +2906,30 @@
         <v>46193</v>
       </c>
       <c r="B35" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C35" s="0" t="s">
         <v>468</v>
       </c>
-      <c r="C35" s="0" t="s">
+      <c r="D35" s="0" t="s">
         <v>469</v>
       </c>
-      <c r="D35" s="0" t="s">
+      <c r="E35" s="0" t="s">
         <v>433</v>
       </c>
-      <c r="E35" s="0">
+      <c r="F35" s="0">
         <v>13</v>
       </c>
-      <c r="F35" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G35" s="0">
+      <c r="G35" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H35" s="0">
         <v>0</v>
       </c>
-      <c r="H35" s="0" t="s">
+      <c r="I35" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I35" s="0" t="s">
+      <c r="J35" s="0" t="s">
         <v>435</v>
       </c>
     </row>
@@ -2827,27 +2938,30 @@
         <v>46195</v>
       </c>
       <c r="B36" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C36" s="0" t="s">
         <v>468</v>
       </c>
-      <c r="C36" s="0" t="s">
+      <c r="D36" s="0" t="s">
         <v>469</v>
       </c>
-      <c r="D36" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E36" s="0">
+      <c r="E36" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F36" s="0">
         <v>6</v>
       </c>
-      <c r="F36" s="0" t="s">
+      <c r="G36" s="0" t="s">
         <v>437</v>
       </c>
-      <c r="G36" s="0">
+      <c r="H36" s="0">
         <v>5</v>
       </c>
-      <c r="H36" s="0" t="s">
+      <c r="I36" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I36" s="0" t="s">
+      <c r="J36" s="0" t="s">
         <v>438</v>
       </c>
     </row>
@@ -2856,27 +2970,30 @@
         <v>46195</v>
       </c>
       <c r="B37" s="0" t="s">
+        <v>471</v>
+      </c>
+      <c r="C37" s="0" t="s">
         <v>468</v>
       </c>
-      <c r="C37" s="0" t="s">
+      <c r="D37" s="0" t="s">
         <v>469</v>
       </c>
-      <c r="D37" s="0" t="s">
+      <c r="E37" s="0" t="s">
         <v>439</v>
       </c>
-      <c r="E37" s="0">
+      <c r="F37" s="0">
         <v>14</v>
       </c>
-      <c r="F37" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G37" s="0">
+      <c r="G37" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H37" s="0">
         <v>3</v>
       </c>
-      <c r="H37" s="0" t="s">
+      <c r="I37" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I37" s="0" t="s">
+      <c r="J37" s="0" t="s">
         <v>440</v>
       </c>
     </row>
@@ -2885,27 +3002,30 @@
         <v>46196</v>
       </c>
       <c r="B38" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C38" s="0" t="s">
         <v>468</v>
       </c>
-      <c r="C38" s="0" t="s">
+      <c r="D38" s="0" t="s">
         <v>469</v>
       </c>
-      <c r="D38" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="E38" s="0">
+      <c r="E38" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="F38" s="0">
         <v>21</v>
       </c>
-      <c r="F38" s="0" t="s">
+      <c r="G38" s="0" t="s">
         <v>441</v>
       </c>
-      <c r="G38" s="0">
+      <c r="H38" s="0">
         <v>1</v>
       </c>
-      <c r="H38" s="0" t="s">
+      <c r="I38" s="0" t="s">
         <v>61</v>
       </c>
-      <c r="I38" s="0" t="s">
+      <c r="J38" s="0" t="s">
         <v>442</v>
       </c>
     </row>
@@ -2914,27 +3034,30 @@
         <v>46196</v>
       </c>
       <c r="B39" s="0" t="s">
+        <v>472</v>
+      </c>
+      <c r="C39" s="0" t="s">
         <v>468</v>
       </c>
-      <c r="C39" s="0" t="s">
+      <c r="D39" s="0" t="s">
         <v>469</v>
       </c>
-      <c r="D39" s="0" t="s">
+      <c r="E39" s="0" t="s">
         <v>436</v>
       </c>
-      <c r="E39" s="0">
+      <c r="F39" s="0">
         <v>6</v>
       </c>
-      <c r="F39" s="0" t="s">
-        <v>369</v>
-      </c>
-      <c r="G39" s="0">
+      <c r="G39" s="0" t="s">
+        <v>369</v>
+      </c>
+      <c r="H39" s="0">
         <v>5</v>
       </c>
-      <c r="H39" s="0" t="s">
+      <c r="I39" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="I39" s="0" t="s">
+      <c r="J39" s="0" t="s">
         <v>443</v>
       </c>
     </row>

</xml_diff>